<commit_message>
Forward curve, market access criterion, criteria chart
</commit_message>
<xml_diff>
--- a/output/ranking.xlsx
+++ b/output/ranking.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,35 +430,55 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>spot</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>forward</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fwd_above_spot</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>carry</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rolldown_bps</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>excess</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>breakeven_bps</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>vol_bps</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sharpe</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>public_market</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>passes</t>
         </is>
@@ -474,20 +494,32 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
+        <v>3.542</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.843</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
         <v>1.1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="G2" t="n">
         <v>30</v>
       </c>
-      <c r="E2" t="n">
+      <c r="H2" t="n">
         <v>1.39</v>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="n">
         <v>143.8</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="b">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -501,20 +533,32 @@
         <v>3</v>
       </c>
       <c r="C3" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.987</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
         <v>1.25</v>
       </c>
-      <c r="D3" t="n">
+      <c r="G3" t="n">
         <v>14.8</v>
       </c>
-      <c r="E3" t="n">
+      <c r="H3" t="n">
         <v>1.54</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="n">
         <v>79.5</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="b">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -528,20 +572,32 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
+        <v>3.825</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.231</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
         <v>1.39</v>
       </c>
-      <c r="D4" t="n">
+      <c r="G4" t="n">
         <v>13.5</v>
       </c>
-      <c r="E4" t="n">
+      <c r="H4" t="n">
         <v>1.78</v>
       </c>
-      <c r="F4" t="n">
+      <c r="I4" t="n">
         <v>61.4</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="b">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -555,20 +611,32 @@
         <v>5</v>
       </c>
       <c r="C5" t="n">
+        <v>3.994</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.673</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
         <v>1.55</v>
       </c>
-      <c r="D5" t="n">
+      <c r="G5" t="n">
         <v>16.9</v>
       </c>
-      <c r="E5" t="n">
+      <c r="H5" t="n">
         <v>2.21</v>
       </c>
-      <c r="F5" t="n">
+      <c r="I5" t="n">
         <v>57.2</v>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="b">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -582,20 +650,32 @@
         <v>6</v>
       </c>
       <c r="C6" t="n">
+        <v>4.115</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4.722</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
         <v>1.68</v>
       </c>
-      <c r="D6" t="n">
+      <c r="G6" t="n">
         <v>12.1</v>
       </c>
-      <c r="E6" t="n">
+      <c r="H6" t="n">
         <v>2.26</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="n">
         <v>46.9</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="b">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -609,20 +689,32 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
+        <v>4.257</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.113</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
         <v>1.82</v>
       </c>
-      <c r="D7" t="n">
+      <c r="G7" t="n">
         <v>14.2</v>
       </c>
-      <c r="E7" t="n">
+      <c r="H7" t="n">
         <v>2.64</v>
       </c>
-      <c r="F7" t="n">
+      <c r="I7" t="n">
         <v>45.7</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="b">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -636,20 +728,32 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
+        <v>4.378</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.229</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
         <v>1.94</v>
       </c>
-      <c r="D8" t="n">
+      <c r="G8" t="n">
         <v>12.1</v>
       </c>
-      <c r="E8" t="n">
+      <c r="H8" t="n">
         <v>2.75</v>
       </c>
-      <c r="F8" t="n">
+      <c r="I8" t="n">
         <v>41</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="b">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -663,20 +767,32 @@
         <v>9</v>
       </c>
       <c r="C9" t="n">
+        <v>4.501</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
         <v>2.06</v>
       </c>
-      <c r="D9" t="n">
+      <c r="G9" t="n">
         <v>12.3</v>
       </c>
-      <c r="E9" t="n">
+      <c r="H9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" t="n">
+      <c r="I9" t="n">
         <v>39.2</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="b">
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -690,20 +806,32 @@
         <v>10</v>
       </c>
       <c r="C10" t="n">
+        <v>4.614</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.637</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
         <v>2.17</v>
       </c>
-      <c r="D10" t="n">
+      <c r="G10" t="n">
         <v>11.3</v>
       </c>
-      <c r="E10" t="n">
+      <c r="H10" t="n">
         <v>3.15</v>
       </c>
-      <c r="F10" t="n">
+      <c r="I10" t="n">
         <v>36.5</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="b">
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -717,20 +845,32 @@
         <v>15</v>
       </c>
       <c r="C11" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.857</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
         <v>2.5</v>
       </c>
-      <c r="D11" t="n">
+      <c r="G11" t="n">
         <v>6.5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="H11" t="n">
         <v>3.37</v>
       </c>
-      <c r="F11" t="n">
+      <c r="I11" t="n">
         <v>25.2</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="b">
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -744,20 +884,32 @@
         <v>2</v>
       </c>
       <c r="C12" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3.525</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
         <v>0.83</v>
       </c>
-      <c r="D12" t="n">
+      <c r="G12" t="n">
         <v>25.4</v>
       </c>
-      <c r="E12" t="n">
+      <c r="H12" t="n">
         <v>1.08</v>
       </c>
-      <c r="F12" t="n">
+      <c r="I12" t="n">
         <v>110.9</v>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="b">
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -771,20 +923,32 @@
         <v>7</v>
       </c>
       <c r="C13" t="n">
+        <v>3.412</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.719</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
         <v>0.97</v>
       </c>
-      <c r="D13" t="n">
+      <c r="G13" t="n">
         <v>5.1</v>
       </c>
-      <c r="E13" t="n">
+      <c r="H13" t="n">
         <v>1.27</v>
       </c>
-      <c r="F13" t="n">
+      <c r="I13" t="n">
         <v>21.8</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="b">
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -798,20 +962,32 @@
         <v>2</v>
       </c>
       <c r="C14" t="n">
+        <v>3.581</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.932</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
         <v>1.14</v>
       </c>
-      <c r="D14" t="n">
+      <c r="G14" t="n">
         <v>35</v>
       </c>
-      <c r="E14" t="n">
+      <c r="H14" t="n">
         <v>1.48</v>
       </c>
-      <c r="F14" t="n">
+      <c r="I14" t="n">
         <v>152.8</v>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="b">
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="b">
         <v>1</v>
       </c>
     </row>
@@ -825,20 +1001,32 @@
         <v>3</v>
       </c>
       <c r="C15" t="n">
+        <v>3.733</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4.038</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
         <v>1.29</v>
       </c>
-      <c r="D15" t="n">
+      <c r="G15" t="n">
         <v>15.2</v>
       </c>
-      <c r="E15" t="n">
+      <c r="H15" t="n">
         <v>1.59</v>
       </c>
-      <c r="F15" t="n">
+      <c r="I15" t="n">
         <v>82.2</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="b">
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -852,20 +1040,32 @@
         <v>4</v>
       </c>
       <c r="C16" t="n">
+        <v>3.852</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
         <v>1.41</v>
       </c>
-      <c r="D16" t="n">
+      <c r="G16" t="n">
         <v>11.9</v>
       </c>
-      <c r="E16" t="n">
+      <c r="H16" t="n">
         <v>1.76</v>
       </c>
-      <c r="F16" t="n">
+      <c r="I16" t="n">
         <v>60.7</v>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="b">
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -879,20 +1079,32 @@
         <v>5</v>
       </c>
       <c r="C17" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.443</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
         <v>1.53</v>
       </c>
-      <c r="D17" t="n">
+      <c r="G17" t="n">
         <v>11.8</v>
       </c>
-      <c r="E17" t="n">
+      <c r="H17" t="n">
         <v>1.98</v>
       </c>
-      <c r="F17" t="n">
+      <c r="I17" t="n">
         <v>51.5</v>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="b">
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="b">
         <v>1</v>
       </c>
     </row>
@@ -906,20 +1118,32 @@
         <v>6</v>
       </c>
       <c r="C18" t="n">
+        <v>4.075</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.602</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
         <v>1.64</v>
       </c>
-      <c r="D18" t="n">
+      <c r="G18" t="n">
         <v>10.5</v>
       </c>
-      <c r="E18" t="n">
+      <c r="H18" t="n">
         <v>2.14</v>
       </c>
-      <c r="F18" t="n">
+      <c r="I18" t="n">
         <v>44.5</v>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="b">
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -933,20 +1157,32 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
+        <v>4.191</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
         <v>1.75</v>
       </c>
-      <c r="D19" t="n">
+      <c r="G19" t="n">
         <v>11.6</v>
       </c>
-      <c r="E19" t="n">
+      <c r="H19" t="n">
         <v>2.42</v>
       </c>
-      <c r="F19" t="n">
+      <c r="I19" t="n">
         <v>42</v>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="b">
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -960,20 +1196,32 @@
         <v>8</v>
       </c>
       <c r="C20" t="n">
+        <v>4.295</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5.026</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
         <v>1.86</v>
       </c>
-      <c r="D20" t="n">
+      <c r="G20" t="n">
         <v>10.4</v>
       </c>
-      <c r="E20" t="n">
+      <c r="H20" t="n">
         <v>2.55</v>
       </c>
-      <c r="F20" t="n">
+      <c r="I20" t="n">
         <v>38</v>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="b">
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -987,20 +1235,32 @@
         <v>9</v>
       </c>
       <c r="C21" t="n">
+        <v>4.393</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
         <v>1.95</v>
       </c>
-      <c r="D21" t="n">
+      <c r="G21" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E21" t="n">
+      <c r="H21" t="n">
         <v>2.7</v>
       </c>
-      <c r="F21" t="n">
+      <c r="I21" t="n">
         <v>35.3</v>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="b">
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1014,20 +1274,32 @@
         <v>10</v>
       </c>
       <c r="C22" t="n">
+        <v>4.488</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5.347</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
         <v>2.05</v>
       </c>
-      <c r="D22" t="n">
+      <c r="G22" t="n">
         <v>9.5</v>
       </c>
-      <c r="E22" t="n">
+      <c r="H22" t="n">
         <v>2.87</v>
       </c>
-      <c r="F22" t="n">
+      <c r="I22" t="n">
         <v>33.3</v>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="b">
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1041,20 +1313,32 @@
         <v>15</v>
       </c>
       <c r="C23" t="n">
+        <v>4.796</v>
+      </c>
+      <c r="D23" t="n">
+        <v>5.662</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
         <v>2.36</v>
       </c>
-      <c r="D23" t="n">
+      <c r="G23" t="n">
         <v>6.2</v>
       </c>
-      <c r="E23" t="n">
+      <c r="H23" t="n">
         <v>3.18</v>
       </c>
-      <c r="F23" t="n">
+      <c r="I23" t="n">
         <v>23.8</v>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="b">
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>